<commit_message>
Update budget — 4/19/2026, 10:24:41 PM
</commit_message>
<xml_diff>
--- a/Monthly-Budget.xlsx
+++ b/Monthly-Budget.xlsx
@@ -785,7 +785,7 @@
         <v>Investments</v>
       </c>
       <c r="B10">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="D10">
         <f>C10-B10</f>
@@ -804,7 +804,7 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="O10">
         <v>0</v>

</xml_diff>